<commit_message>
feat: implement shared plan 52
</commit_message>
<xml_diff>
--- a/data/source/official-cti-2025/cti-basic-000040499069.xlsx
+++ b/data/source/official-cti-2025/cti-basic-000040499069.xlsx
@@ -1,27 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://digitalgojp.sharepoint.com/sites/MIC_FS00007/DocLib2/10消費指標/10【中分類】結果の公表関係/_検討中/02【小分類：20370331廃】（検討中）2026年度消費動向指数公表関係/2025年基準/11_インターネット関係/e-stat/01_公表統計表作成/01_CTI/統計表/月次/202607/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://digitalgojp.sharepoint.com/sites/MIC_FS00007/DocLib2/10消費指標/10【中分類】結果の公表関係/_検討中/02【小分類：20370331廃】（検討中）2026年度消費動向指数公表関係/2025年基準/11_インターネット関係/e-stat/01_公表統計表作成/01_CTI/統計表/月次/202608/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="248" documentId="13_ncr:1_{9D012BE2-D796-40B0-B3A3-B89464F745C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{322DB028-8A51-4E0F-9B7D-987400DE0426}"/>
+  <xr:revisionPtr revIDLastSave="266" documentId="13_ncr:1_{9D012BE2-D796-40B0-B3A3-B89464F745C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E1089E0B-8558-42D6-8EBA-DC9C2601CC6E}"/>
   <bookViews>
-    <workbookView xWindow="1572" yWindow="1092" windowWidth="21468" windowHeight="13308" tabRatio="783" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30840" yWindow="2115" windowWidth="23475" windowHeight="14205" tabRatio="783" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="総・月(原)" sheetId="69" r:id="rId1"/>
-    <sheet name="財サ・総・月(原)" sheetId="70" r:id="rId2"/>
+    <sheet name="総・月(原)" sheetId="73" r:id="rId1"/>
+    <sheet name="財サ・総・月(原)" sheetId="74" r:id="rId2"/>
     <sheet name="総・四(原)" sheetId="51" r:id="rId3"/>
     <sheet name="財サ・総・四(原)" sheetId="52" r:id="rId4"/>
     <sheet name="総・年" sheetId="32" r:id="rId5"/>
     <sheet name="財サ・総・年" sheetId="33" r:id="rId6"/>
     <sheet name="総・年度" sheetId="44" r:id="rId7"/>
-    <sheet name="総(勤)・月(原)" sheetId="71" r:id="rId8"/>
-    <sheet name="財サ・総(勤)・月(原)" sheetId="72" r:id="rId9"/>
+    <sheet name="総(勤)・月(原)" sheetId="75" r:id="rId8"/>
+    <sheet name="財サ・総(勤)・月(原)" sheetId="76" r:id="rId9"/>
     <sheet name="総(勤)・四(原)" sheetId="55" r:id="rId10"/>
     <sheet name="財サ・総(勤)・四(原)" sheetId="56" r:id="rId11"/>
     <sheet name="総(勤)・年" sheetId="38" r:id="rId12"/>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4435" uniqueCount="556">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4455" uniqueCount="558">
   <si>
     <t>統計名：</t>
   </si>
@@ -2070,6 +2070,13 @@
   <si>
     <t>注4. 2020年基準改定において「授業料等」及び「仕送り金」の取り扱いを変更したため、2019年以前の「その他の消費支出」は「-」としている。詳細は「世帯消費動向指数（CTIミクロ）の推定方法」参照。</t>
   </si>
+  <si>
+    <t xml:space="preserve">202608B     </t>
+  </si>
+  <si>
+    <t>2026年8月</t>
+    <phoneticPr fontId="2"/>
+  </si>
 </sst>
 </file>
 
@@ -2677,8 +2684,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F871B57D-0C61-4461-9655-6C01968FABD4}">
-  <dimension ref="A1:AF132"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DBF20B43-A9BD-47FB-9413-126308E2E642}">
+  <dimension ref="A1:AF133"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="13.65" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="5" width="0" style="1" hidden="1" customWidth="1"/>
@@ -13327,72 +13334,162 @@
         <v>13.238</v>
       </c>
     </row>
-    <row r="125" spans="1:31" ht="13.65" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F125" s="12"/>
-      <c r="H125" s="25" t="s">
-        <v>24</v>
-      </c>
-      <c r="I125" s="26"/>
-      <c r="J125" s="26"/>
-      <c r="K125" s="26"/>
-      <c r="L125" s="26"/>
-      <c r="M125" s="26"/>
-      <c r="N125" s="26"/>
-      <c r="O125" s="26"/>
-      <c r="P125" s="26"/>
-      <c r="Q125" s="26"/>
-      <c r="R125" s="26"/>
-      <c r="S125" s="26"/>
-      <c r="T125" s="26"/>
-      <c r="U125" s="26"/>
-      <c r="V125" s="26"/>
-      <c r="W125" s="26"/>
-      <c r="X125" s="26"/>
-      <c r="Y125" s="26"/>
-      <c r="Z125" s="26"/>
-      <c r="AA125" s="26"/>
-      <c r="AB125" s="26"/>
-      <c r="AC125" s="26"/>
-      <c r="AD125" s="26"/>
-      <c r="AE125" s="26"/>
+    <row r="125" spans="1:31" ht="14.1" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A125" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="B125" s="13" t="s">
+        <v>556</v>
+      </c>
+      <c r="C125" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="D125" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="E125" s="13"/>
+      <c r="F125" s="4">
+        <v>1</v>
+      </c>
+      <c r="H125" s="14">
+        <v>2026000808</v>
+      </c>
+      <c r="I125" s="9" t="s">
+        <v>557</v>
+      </c>
+      <c r="J125" s="10">
+        <v>100.1177</v>
+      </c>
+      <c r="K125" s="11">
+        <v>31.169</v>
+      </c>
+      <c r="L125" s="11">
+        <v>7.9481999999999999</v>
+      </c>
+      <c r="M125" s="11">
+        <v>6.1577000000000002</v>
+      </c>
+      <c r="N125" s="11">
+        <v>4.5503999999999998</v>
+      </c>
+      <c r="O125" s="11">
+        <v>2.5188000000000001</v>
+      </c>
+      <c r="P125" s="11">
+        <v>4.9458000000000002</v>
+      </c>
+      <c r="Q125" s="11">
+        <v>15.628399999999999</v>
+      </c>
+      <c r="R125" s="11">
+        <v>1.6687000000000001</v>
+      </c>
+      <c r="S125" s="11">
+        <v>11.393800000000001</v>
+      </c>
+      <c r="T125" s="11">
+        <v>14.1366</v>
+      </c>
+      <c r="U125" s="11">
+        <v>97.675799999999995</v>
+      </c>
+      <c r="V125" s="11">
+        <v>30.027899999999999</v>
+      </c>
+      <c r="W125" s="11">
+        <v>7.7167000000000003</v>
+      </c>
+      <c r="X125" s="11">
+        <v>6.335</v>
+      </c>
+      <c r="Y125" s="11">
+        <v>4.3009000000000004</v>
+      </c>
+      <c r="Z125" s="11">
+        <v>2.5163000000000002</v>
+      </c>
+      <c r="AA125" s="11">
+        <v>4.7877999999999998</v>
+      </c>
+      <c r="AB125" s="11">
+        <v>15.1584</v>
+      </c>
+      <c r="AC125" s="11">
+        <v>1.7492000000000001</v>
+      </c>
+      <c r="AD125" s="11">
+        <v>10.9872</v>
+      </c>
+      <c r="AE125" s="11">
+        <v>13.7918</v>
+      </c>
     </row>
     <row r="126" spans="1:31" ht="13.65" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F126" s="12"/>
-      <c r="H126" s="27" t="s">
-        <v>533</v>
-      </c>
+      <c r="H126" s="25" t="s">
+        <v>24</v>
+      </c>
+      <c r="I126" s="26"/>
+      <c r="J126" s="26"/>
+      <c r="K126" s="26"/>
+      <c r="L126" s="26"/>
+      <c r="M126" s="26"/>
+      <c r="N126" s="26"/>
+      <c r="O126" s="26"/>
+      <c r="P126" s="26"/>
+      <c r="Q126" s="26"/>
+      <c r="R126" s="26"/>
+      <c r="S126" s="26"/>
+      <c r="T126" s="26"/>
+      <c r="U126" s="26"/>
+      <c r="V126" s="26"/>
+      <c r="W126" s="26"/>
+      <c r="X126" s="26"/>
+      <c r="Y126" s="26"/>
+      <c r="Z126" s="26"/>
+      <c r="AA126" s="26"/>
+      <c r="AB126" s="26"/>
+      <c r="AC126" s="26"/>
+      <c r="AD126" s="26"/>
+      <c r="AE126" s="26"/>
     </row>
     <row r="127" spans="1:31" ht="13.65" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F127" s="12"/>
       <c r="H127" s="27" t="s">
-        <v>25</v>
+        <v>533</v>
       </c>
     </row>
     <row r="128" spans="1:31" ht="13.65" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F128" s="12"/>
-      <c r="H128" s="28" t="s">
-        <v>555</v>
+      <c r="H128" s="27" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="129" spans="6:8" ht="13.65" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F129" s="12"/>
       <c r="H129" s="28" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
     </row>
     <row r="130" spans="6:8" ht="13.65" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F130" s="12"/>
-      <c r="H130" s="27" t="s">
+      <c r="H130" s="28" t="s">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="131" spans="6:8" ht="13.65" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F131" s="12"/>
+      <c r="H131" s="27" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="131" spans="6:8" ht="13.65" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F131" s="5"/>
-    </row>
     <row r="132" spans="6:8" ht="13.65" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F132"/>
-      <c r="G132"/>
-      <c r="H132"/>
+      <c r="F132" s="5"/>
+    </row>
+    <row r="133" spans="6:8" ht="13.65" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F133"/>
+      <c r="G133"/>
+      <c r="H133"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2"/>
@@ -13400,7 +13497,7 @@
   <pageMargins left="0.39370078740157483" right="0" top="0.59055118110236227" bottom="0" header="0.39370078740157483" footer="0.39370078740157483"/>
   <pageSetup paperSize="9" fitToWidth="0" fitToHeight="0" pageOrder="overThenDown" orientation="portrait" r:id="rId1"/>
   <rowBreaks count="1" manualBreakCount="1">
-    <brk id="131" max="16383" man="1"/>
+    <brk id="132" max="16383" man="1"/>
   </rowBreaks>
   <colBreaks count="1" manualBreakCount="1">
     <brk id="32" max="1048575" man="1"/>
@@ -27560,8 +27657,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB829D31-D49D-4819-A91F-40EB1260783E}">
-  <dimension ref="A1:V94"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{552314E1-1D7B-459B-B635-944A9653C544}">
+  <dimension ref="A1:V95"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="13.65" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="5" width="0" style="1" hidden="1" customWidth="1"/>
@@ -32482,52 +32579,112 @@
         <v>38.728299999999997</v>
       </c>
     </row>
-    <row r="89" spans="1:21" ht="13.65" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F89" s="12"/>
-      <c r="H89" s="32" t="s">
-        <v>24</v>
-      </c>
-      <c r="I89" s="26"/>
-      <c r="J89" s="25"/>
-      <c r="K89" s="26"/>
-      <c r="L89" s="26"/>
-      <c r="M89" s="26"/>
-      <c r="N89" s="26"/>
-      <c r="O89" s="26"/>
-      <c r="P89" s="26"/>
-      <c r="Q89" s="26"/>
-      <c r="R89" s="26"/>
-      <c r="S89" s="26"/>
-      <c r="T89" s="26"/>
-      <c r="U89" s="26"/>
+    <row r="89" spans="1:21" ht="14.1" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A89" s="13" t="s">
+        <v>149</v>
+      </c>
+      <c r="B89" s="13" t="s">
+        <v>556</v>
+      </c>
+      <c r="C89" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="D89" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="E89" s="13"/>
+      <c r="F89" s="4">
+        <v>1</v>
+      </c>
+      <c r="H89" s="14">
+        <v>2026000808</v>
+      </c>
+      <c r="I89" s="9" t="s">
+        <v>557</v>
+      </c>
+      <c r="J89" s="10">
+        <v>94.974900000000005</v>
+      </c>
+      <c r="K89" s="11">
+        <v>53.570700000000002</v>
+      </c>
+      <c r="L89" s="11">
+        <v>8.0277999999999992</v>
+      </c>
+      <c r="M89" s="11">
+        <v>6.5312999999999999</v>
+      </c>
+      <c r="N89" s="11">
+        <v>39.011600000000001</v>
+      </c>
+      <c r="O89" s="11">
+        <v>41.404600000000002</v>
+      </c>
+      <c r="P89" s="11">
+        <v>92.6584</v>
+      </c>
+      <c r="Q89" s="11">
+        <v>52.213200000000001</v>
+      </c>
+      <c r="R89" s="11">
+        <v>7.7789000000000001</v>
+      </c>
+      <c r="S89" s="11">
+        <v>6.3906999999999998</v>
+      </c>
+      <c r="T89" s="11">
+        <v>38.023000000000003</v>
+      </c>
+      <c r="U89" s="11">
+        <v>40.473700000000001</v>
+      </c>
     </row>
     <row r="90" spans="1:21" ht="13.65" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F90" s="12"/>
-      <c r="H90" s="34" t="s">
-        <v>533</v>
-      </c>
-      <c r="J90" s="27"/>
+      <c r="H90" s="32" t="s">
+        <v>24</v>
+      </c>
+      <c r="I90" s="26"/>
+      <c r="J90" s="25"/>
+      <c r="K90" s="26"/>
+      <c r="L90" s="26"/>
+      <c r="M90" s="26"/>
+      <c r="N90" s="26"/>
+      <c r="O90" s="26"/>
+      <c r="P90" s="26"/>
+      <c r="Q90" s="26"/>
+      <c r="R90" s="26"/>
+      <c r="S90" s="26"/>
+      <c r="T90" s="26"/>
+      <c r="U90" s="26"/>
     </row>
     <row r="91" spans="1:21" ht="13.65" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F91" s="12"/>
       <c r="H91" s="34" t="s">
-        <v>150</v>
+        <v>533</v>
       </c>
       <c r="J91" s="27"/>
     </row>
     <row r="92" spans="1:21" ht="13.65" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F92" s="12"/>
       <c r="H92" s="34" t="s">
+        <v>150</v>
+      </c>
+      <c r="J92" s="27"/>
+    </row>
+    <row r="93" spans="1:21" ht="13.65" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F93" s="12"/>
+      <c r="H93" s="34" t="s">
         <v>449</v>
       </c>
     </row>
-    <row r="93" spans="1:21" ht="13.65" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F93" s="5"/>
-    </row>
     <row r="94" spans="1:21" ht="13.65" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F94"/>
-      <c r="G94"/>
-      <c r="H94"/>
+      <c r="F94" s="5"/>
+    </row>
+    <row r="95" spans="1:21" ht="13.65" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F95"/>
+      <c r="G95"/>
+      <c r="H95"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2"/>
@@ -32535,7 +32692,7 @@
   <pageMargins left="0.39370078740157483" right="0" top="0.59055118110236227" bottom="0" header="0.39370078740157483" footer="0.39370078740157483"/>
   <pageSetup paperSize="9" fitToWidth="0" fitToHeight="0" pageOrder="overThenDown" orientation="portrait" r:id="rId1"/>
   <rowBreaks count="1" manualBreakCount="1">
-    <brk id="93" max="16383" man="1"/>
+    <brk id="94" max="16383" man="1"/>
   </rowBreaks>
   <colBreaks count="1" manualBreakCount="1">
     <brk id="22" max="1048575" man="1"/>
@@ -47610,8 +47767,8 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7578AD3-CD40-4422-8EC6-69AC56FE3916}">
-  <dimension ref="A1:AF132"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1646A248-2C0C-40A9-8B03-0E504BAC53DF}">
+  <dimension ref="A1:AF133"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="13.65" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="5" width="0" style="1" hidden="1" customWidth="1"/>
@@ -58259,55 +58416,137 @@
         <v>12.9513</v>
       </c>
     </row>
-    <row r="125" spans="1:31" ht="13.65" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F125" s="12"/>
-      <c r="H125" s="25" t="s">
-        <v>24</v>
-      </c>
-      <c r="I125" s="26"/>
-      <c r="J125" s="25"/>
-      <c r="K125" s="26"/>
-      <c r="L125" s="26"/>
-      <c r="M125" s="26"/>
-      <c r="N125" s="26"/>
-      <c r="O125" s="26"/>
-      <c r="P125" s="26"/>
-      <c r="Q125" s="26"/>
-      <c r="R125" s="26"/>
-      <c r="S125" s="26"/>
-      <c r="T125" s="26"/>
-      <c r="U125" s="25"/>
-      <c r="V125" s="26"/>
-      <c r="W125" s="26"/>
-      <c r="X125" s="26"/>
-      <c r="Y125" s="26"/>
-      <c r="Z125" s="26"/>
-      <c r="AA125" s="26"/>
-      <c r="AB125" s="26"/>
-      <c r="AC125" s="26"/>
-      <c r="AD125" s="26"/>
-      <c r="AE125" s="26"/>
+    <row r="125" spans="1:31" ht="14.1" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A125" s="13" t="s">
+        <v>137</v>
+      </c>
+      <c r="B125" s="13" t="s">
+        <v>556</v>
+      </c>
+      <c r="C125" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="D125" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="E125" s="13"/>
+      <c r="F125" s="4">
+        <v>1</v>
+      </c>
+      <c r="H125" s="14">
+        <v>2026000808</v>
+      </c>
+      <c r="I125" s="9" t="s">
+        <v>557</v>
+      </c>
+      <c r="J125" s="11">
+        <v>97.554100000000005</v>
+      </c>
+      <c r="K125" s="11">
+        <v>29.527899999999999</v>
+      </c>
+      <c r="L125" s="11">
+        <v>7.9931999999999999</v>
+      </c>
+      <c r="M125" s="11">
+        <v>5.5591999999999997</v>
+      </c>
+      <c r="N125" s="11">
+        <v>4.1708999999999996</v>
+      </c>
+      <c r="O125" s="11">
+        <v>2.6738</v>
+      </c>
+      <c r="P125" s="11">
+        <v>4.1024000000000003</v>
+      </c>
+      <c r="Q125" s="11">
+        <v>16.845300000000002</v>
+      </c>
+      <c r="R125" s="11">
+        <v>2.0596999999999999</v>
+      </c>
+      <c r="S125" s="11">
+        <v>11.702999999999999</v>
+      </c>
+      <c r="T125" s="11">
+        <v>12.918699999999999</v>
+      </c>
+      <c r="U125" s="11">
+        <v>95.174700000000001</v>
+      </c>
+      <c r="V125" s="11">
+        <v>28.446899999999999</v>
+      </c>
+      <c r="W125" s="11">
+        <v>7.7603999999999997</v>
+      </c>
+      <c r="X125" s="11">
+        <v>5.7194000000000003</v>
+      </c>
+      <c r="Y125" s="11">
+        <v>3.9422000000000001</v>
+      </c>
+      <c r="Z125" s="11">
+        <v>2.6711</v>
+      </c>
+      <c r="AA125" s="11">
+        <v>3.9714</v>
+      </c>
+      <c r="AB125" s="11">
+        <v>16.338799999999999</v>
+      </c>
+      <c r="AC125" s="11">
+        <v>2.1589999999999998</v>
+      </c>
+      <c r="AD125" s="11">
+        <v>11.285500000000001</v>
+      </c>
+      <c r="AE125" s="11">
+        <v>12.6036</v>
+      </c>
     </row>
     <row r="126" spans="1:31" ht="13.65" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F126" s="12"/>
-      <c r="H126" s="27" t="s">
-        <v>533</v>
-      </c>
-      <c r="J126" s="27"/>
-      <c r="U126" s="27"/>
+      <c r="H126" s="25" t="s">
+        <v>24</v>
+      </c>
+      <c r="I126" s="26"/>
+      <c r="J126" s="25"/>
+      <c r="K126" s="26"/>
+      <c r="L126" s="26"/>
+      <c r="M126" s="26"/>
+      <c r="N126" s="26"/>
+      <c r="O126" s="26"/>
+      <c r="P126" s="26"/>
+      <c r="Q126" s="26"/>
+      <c r="R126" s="26"/>
+      <c r="S126" s="26"/>
+      <c r="T126" s="26"/>
+      <c r="U126" s="25"/>
+      <c r="V126" s="26"/>
+      <c r="W126" s="26"/>
+      <c r="X126" s="26"/>
+      <c r="Y126" s="26"/>
+      <c r="Z126" s="26"/>
+      <c r="AA126" s="26"/>
+      <c r="AB126" s="26"/>
+      <c r="AC126" s="26"/>
+      <c r="AD126" s="26"/>
+      <c r="AE126" s="26"/>
     </row>
     <row r="127" spans="1:31" ht="13.65" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F127" s="12"/>
       <c r="H127" s="27" t="s">
-        <v>25</v>
-      </c>
-      <c r="J127" s="28"/>
-      <c r="U127" s="28"/>
+        <v>533</v>
+      </c>
+      <c r="J127" s="27"/>
+      <c r="U127" s="27"/>
     </row>
     <row r="128" spans="1:31" ht="13.65" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F128" s="12"/>
-      <c r="H128" s="28" t="s">
-        <v>555</v>
+      <c r="H128" s="27" t="s">
+        <v>25</v>
       </c>
       <c r="J128" s="28"/>
       <c r="U128" s="28"/>
@@ -58315,22 +58554,28 @@
     <row r="129" spans="6:8" ht="13.65" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F129" s="12"/>
       <c r="H129" s="28" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
     </row>
     <row r="130" spans="6:8" ht="13.65" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F130" s="12"/>
-      <c r="H130" s="27" t="s">
+      <c r="H130" s="28" t="s">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="131" spans="6:8" ht="13.65" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F131" s="12"/>
+      <c r="H131" s="27" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="131" spans="6:8" ht="13.65" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F131" s="5"/>
-    </row>
     <row r="132" spans="6:8" ht="13.65" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F132"/>
-      <c r="G132"/>
-      <c r="H132"/>
+      <c r="F132" s="5"/>
+    </row>
+    <row r="133" spans="6:8" ht="13.65" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F133"/>
+      <c r="G133"/>
+      <c r="H133"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2"/>
@@ -58338,7 +58583,7 @@
   <pageMargins left="0.39370078740157483" right="0" top="0.59055118110236227" bottom="0" header="0.39370078740157483" footer="0.39370078740157483"/>
   <pageSetup paperSize="9" fitToWidth="0" fitToHeight="0" pageOrder="overThenDown" orientation="portrait" r:id="rId1"/>
   <rowBreaks count="1" manualBreakCount="1">
-    <brk id="131" max="16383" man="1"/>
+    <brk id="132" max="16383" man="1"/>
   </rowBreaks>
   <colBreaks count="1" manualBreakCount="1">
     <brk id="32" max="1048575" man="1"/>
@@ -58347,8 +58592,8 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00862E8F-7B68-458A-955C-AF4250AC8ECC}">
-  <dimension ref="A1:V94"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32980567-59B1-4F06-9A0A-39D63FDBF5AE}">
+  <dimension ref="A1:V95"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="13.65" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="5" width="0" style="1" hidden="1" customWidth="1"/>
@@ -63269,53 +63514,113 @@
         <v>40.025199999999998</v>
       </c>
     </row>
-    <row r="89" spans="1:21" ht="13.65" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F89" s="12"/>
-      <c r="H89" s="32" t="s">
-        <v>24</v>
-      </c>
-      <c r="I89" s="26"/>
-      <c r="J89" s="26"/>
-      <c r="K89" s="26"/>
-      <c r="L89" s="26"/>
-      <c r="M89" s="26"/>
-      <c r="N89" s="26"/>
-      <c r="O89" s="26"/>
-      <c r="P89" s="26"/>
-      <c r="Q89" s="26"/>
-      <c r="R89" s="26"/>
-      <c r="S89" s="26"/>
-      <c r="T89" s="26"/>
-      <c r="U89" s="25"/>
+    <row r="89" spans="1:21" ht="14.1" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A89" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="B89" s="13" t="s">
+        <v>556</v>
+      </c>
+      <c r="C89" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="D89" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="E89" s="13"/>
+      <c r="F89" s="4">
+        <v>1</v>
+      </c>
+      <c r="H89" s="14">
+        <v>2026000808</v>
+      </c>
+      <c r="I89" s="9" t="s">
+        <v>557</v>
+      </c>
+      <c r="J89" s="11">
+        <v>92.969300000000004</v>
+      </c>
+      <c r="K89" s="11">
+        <v>50.586100000000002</v>
+      </c>
+      <c r="L89" s="11">
+        <v>7.9016999999999999</v>
+      </c>
+      <c r="M89" s="11">
+        <v>6.8587999999999996</v>
+      </c>
+      <c r="N89" s="11">
+        <v>35.825200000000002</v>
+      </c>
+      <c r="O89" s="11">
+        <v>42.383200000000002</v>
+      </c>
+      <c r="P89" s="11">
+        <v>90.701800000000006</v>
+      </c>
+      <c r="Q89" s="11">
+        <v>49.304200000000002</v>
+      </c>
+      <c r="R89" s="11">
+        <v>7.6566999999999998</v>
+      </c>
+      <c r="S89" s="11">
+        <v>6.7111999999999998</v>
+      </c>
+      <c r="T89" s="11">
+        <v>34.917299999999997</v>
+      </c>
+      <c r="U89" s="11">
+        <v>41.430300000000003</v>
+      </c>
     </row>
     <row r="90" spans="1:21" ht="13.65" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F90" s="12"/>
-      <c r="H90" s="34" t="s">
-        <v>533</v>
-      </c>
-      <c r="J90" s="27"/>
-      <c r="U90" s="27"/>
+      <c r="H90" s="32" t="s">
+        <v>24</v>
+      </c>
+      <c r="I90" s="26"/>
+      <c r="J90" s="26"/>
+      <c r="K90" s="26"/>
+      <c r="L90" s="26"/>
+      <c r="M90" s="26"/>
+      <c r="N90" s="26"/>
+      <c r="O90" s="26"/>
+      <c r="P90" s="26"/>
+      <c r="Q90" s="26"/>
+      <c r="R90" s="26"/>
+      <c r="S90" s="26"/>
+      <c r="T90" s="26"/>
+      <c r="U90" s="25"/>
     </row>
     <row r="91" spans="1:21" ht="13.65" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F91" s="12"/>
       <c r="H91" s="34" t="s">
-        <v>150</v>
+        <v>533</v>
       </c>
       <c r="J91" s="27"/>
+      <c r="U91" s="27"/>
     </row>
     <row r="92" spans="1:21" ht="13.65" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F92" s="12"/>
       <c r="H92" s="34" t="s">
+        <v>150</v>
+      </c>
+      <c r="J92" s="27"/>
+    </row>
+    <row r="93" spans="1:21" ht="13.65" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F93" s="12"/>
+      <c r="H93" s="34" t="s">
         <v>449</v>
       </c>
     </row>
-    <row r="93" spans="1:21" ht="13.65" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F93" s="5"/>
-    </row>
     <row r="94" spans="1:21" ht="13.65" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F94"/>
-      <c r="G94"/>
-      <c r="H94"/>
+      <c r="F94" s="5"/>
+    </row>
+    <row r="95" spans="1:21" ht="13.65" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F95"/>
+      <c r="G95"/>
+      <c r="H95"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2"/>
@@ -63323,7 +63628,7 @@
   <pageMargins left="0.39370078740157483" right="0" top="0.59055118110236227" bottom="0" header="0.39370078740157483" footer="0.39370078740157483"/>
   <pageSetup paperSize="9" fitToWidth="0" fitToHeight="0" pageOrder="overThenDown" orientation="portrait" r:id="rId1"/>
   <rowBreaks count="1" manualBreakCount="1">
-    <brk id="93" max="16383" man="1"/>
+    <brk id="94" max="16383" man="1"/>
   </rowBreaks>
   <colBreaks count="1" manualBreakCount="1">
     <brk id="22" max="1048575" man="1"/>
@@ -63587,16 +63892,16 @@
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E070D91A-69A4-48CD-A0B7-3F0C9F4E76A7}">
   <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="ea419855-74cd-451e-b55c-dc846f6a406d"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="cb2765f4-8816-4b89-8f0e-f2ffa45504c3"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="ea419855-74cd-451e-b55c-dc846f6a406d"/>
-    <ds:schemaRef ds:uri="cb2765f4-8816-4b89-8f0e-f2ffa45504c3"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>